<commit_message>
Rescore comfort ratings in a single pass for cross-city consistency
</commit_message>
<xml_diff>
--- a/metravel_transport_dataset.xlsx
+++ b/metravel_transport_dataset.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="398" uniqueCount="211">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="398" uniqueCount="212">
   <si>
     <t xml:space="preserve">MeTravel — Transport Price Dataset</t>
   </si>
@@ -595,6 +595,9 @@
   </si>
   <si>
     <t xml:space="preserve">MRT East-West Line</t>
+  </si>
+  <si>
+    <t xml:space="preserve">05:31</t>
   </si>
   <si>
     <t xml:space="preserve">23:18</t>
@@ -670,7 +673,7 @@
     <numFmt numFmtId="166" formatCode="#,##0.00"/>
     <numFmt numFmtId="167" formatCode="@"/>
   </numFmts>
-  <fonts count="16">
+  <fonts count="15">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -751,14 +754,6 @@
       <color rgb="FFC00000"/>
       <name val="Arial"/>
       <family val="2"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="10"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Arial"/>
-      <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
@@ -876,48 +871,44 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="33">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -925,7 +916,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -941,15 +932,15 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="13" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="13" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -961,7 +952,7 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="13" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="7" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -969,7 +960,7 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="13" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="7" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -985,19 +976,15 @@
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="7" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="13" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="13" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1005,15 +992,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1357,210 +1344,210 @@
   <dimension ref="A1:B39"/>
   <sheetFormatPr defaultColWidth="8.66796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="46"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="95"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="95"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="4" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="5" t="s">
+      <c r="A6" s="4" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="5" t="s">
+      <c r="A7" s="4" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="5" t="s">
+      <c r="A8" s="4" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="5" t="s">
+      <c r="A9" s="4" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="4" t="s">
+      <c r="A11" s="3" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="6" t="s">
+      <c r="A12" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="B12" s="5" t="s">
+      <c r="B12" s="4" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="6" t="s">
+      <c r="A13" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="B13" s="4" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="6" t="s">
+      <c r="A14" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="B14" s="5" t="s">
+      <c r="B14" s="4" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="6" t="s">
+      <c r="A15" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="B15" s="5" t="s">
+      <c r="B15" s="4" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="6" t="s">
+      <c r="A16" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="B16" s="5" t="s">
+      <c r="B16" s="4" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="6" t="s">
+      <c r="A17" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="B17" s="5" t="s">
+      <c r="B17" s="4" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="6" t="s">
+      <c r="A18" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="B18" s="5" t="s">
+      <c r="B18" s="4" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="6" t="s">
+      <c r="A19" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="B19" s="5" t="s">
+      <c r="B19" s="4" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="6" t="s">
+      <c r="A20" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="B20" s="5" t="s">
+      <c r="B20" s="4" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="6" t="s">
+      <c r="A21" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="B21" s="5" t="s">
+      <c r="B21" s="4" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="6" t="s">
+      <c r="A22" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="B22" s="5" t="s">
+      <c r="B22" s="4" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="4" t="s">
+      <c r="A24" s="3" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="5" t="s">
+      <c r="A25" s="4" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="5" t="s">
+      <c r="A26" s="4" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="5" t="s">
+      <c r="A27" s="4" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="5" t="s">
+      <c r="A28" s="4" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="5" t="s">
+      <c r="A29" s="4" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="4" t="s">
+      <c r="A31" s="3" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="5" t="s">
+      <c r="A32" s="4" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="5" t="s">
+      <c r="A33" s="4" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="5" t="s">
+      <c r="A34" s="4" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="5" t="s">
+      <c r="A35" s="4" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="5" t="s">
+      <c r="A36" s="4" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="4" t="s">
+      <c r="A38" s="3" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="5" t="s">
+      <c r="A39" s="4" t="s">
         <v>44</v>
       </c>
     </row>
@@ -1583,122 +1570,122 @@
   <dimension ref="A1:C14"/>
   <sheetFormatPr defaultColWidth="8.66796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="16"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="2" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="7" t="s">
+      <c r="A4" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="B4" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="C4" s="6" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="8" t="s">
+      <c r="A5" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="B5" s="8" t="s">
+      <c r="B5" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="C5" s="9" t="n">
+      <c r="C5" s="8" t="n">
         <v>780</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="8" t="s">
+      <c r="A6" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="B6" s="8" t="s">
+      <c r="B6" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="C6" s="9" t="n">
+      <c r="C6" s="8" t="n">
         <v>19</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="8" t="s">
+      <c r="A7" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="B7" s="8" t="s">
+      <c r="B7" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="C7" s="9" t="n">
+      <c r="C7" s="8" t="n">
         <v>175</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="8" t="s">
+      <c r="A8" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="B8" s="8" t="s">
+      <c r="B8" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="C8" s="9" t="n">
+      <c r="C8" s="8" t="n">
         <v>19500</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="8" t="s">
+      <c r="A9" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="B9" s="8" t="s">
+      <c r="B9" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="C9" s="9" t="n">
+      <c r="C9" s="8" t="n">
         <v>800</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="8" t="s">
+      <c r="A10" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="B10" s="8" t="s">
+      <c r="B10" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="C10" s="9" t="n">
+      <c r="C10" s="8" t="n">
         <v>25500</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="8" t="s">
+      <c r="A11" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="B11" s="8" t="s">
+      <c r="B11" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="C11" s="9" t="n">
+      <c r="C11" s="8" t="n">
         <v>5900</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="8" t="s">
+      <c r="A12" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="B12" s="8" t="s">
+      <c r="B12" s="7" t="s">
         <v>65</v>
       </c>
-      <c r="C12" s="9" t="n">
+      <c r="C12" s="8" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="10" t="s">
+      <c r="A14" s="9" t="s">
         <v>66</v>
       </c>
     </row>
@@ -1721,1521 +1708,1522 @@
   <dimension ref="A1:Y19"/>
   <sheetFormatPr defaultColWidth="8.66796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="1" style="1" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="9" style="1" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="13" style="1" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="15" style="1" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="1" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="1" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="1" width="55"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="1" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="1" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="22" style="1" width="45"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="23" min="23" style="1" width="40"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="25" min="24" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="1" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="9" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="13" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="20.16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="17.16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="0" width="55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="22" style="0" width="45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="23" min="23" style="0" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="25" min="24" style="0" width="14"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="B1" s="11" t="s">
+      <c r="B1" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="C1" s="11" t="s">
+      <c r="C1" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="D1" s="11" t="s">
+      <c r="D1" s="10" t="s">
         <v>69</v>
       </c>
-      <c r="E1" s="11" t="s">
+      <c r="E1" s="10" t="s">
         <v>70</v>
       </c>
-      <c r="F1" s="11" t="s">
+      <c r="F1" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="G1" s="11" t="s">
+      <c r="G1" s="10" t="s">
         <v>71</v>
       </c>
-      <c r="H1" s="11" t="s">
+      <c r="H1" s="10" t="s">
         <v>72</v>
       </c>
-      <c r="I1" s="11" t="s">
+      <c r="I1" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="J1" s="11" t="s">
+      <c r="J1" s="10" t="s">
         <v>74</v>
       </c>
-      <c r="K1" s="11" t="s">
+      <c r="K1" s="10" t="s">
         <v>75</v>
       </c>
-      <c r="L1" s="11" t="s">
+      <c r="L1" s="10" t="s">
         <v>76</v>
       </c>
-      <c r="M1" s="11" t="s">
+      <c r="M1" s="10" t="s">
         <v>77</v>
       </c>
-      <c r="N1" s="11" t="s">
+      <c r="N1" s="10" t="s">
         <v>78</v>
       </c>
-      <c r="O1" s="11" t="s">
+      <c r="O1" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="P1" s="11" t="s">
+      <c r="P1" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="Q1" s="11" t="s">
+      <c r="Q1" s="10" t="s">
         <v>79</v>
       </c>
-      <c r="R1" s="11" t="s">
+      <c r="R1" s="10" t="s">
         <v>80</v>
       </c>
-      <c r="S1" s="11" t="s">
+      <c r="S1" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="T1" s="11" t="s">
+      <c r="T1" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="U1" s="11" t="s">
+      <c r="U1" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="V1" s="11" t="s">
+      <c r="V1" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="W1" s="11" t="s">
+      <c r="W1" s="10" t="s">
         <v>81</v>
       </c>
-      <c r="X1" s="11" t="s">
+      <c r="X1" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="Y1" s="12" t="s">
+      <c r="Y1" s="11" t="s">
         <v>82</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="13" t="s">
+      <c r="A2" s="12" t="s">
         <v>83</v>
       </c>
-      <c r="B2" s="13" t="s">
+      <c r="B2" s="12" t="s">
         <v>84</v>
       </c>
-      <c r="C2" s="13" t="s">
+      <c r="C2" s="12" t="s">
         <v>85</v>
       </c>
-      <c r="D2" s="13" t="s">
+      <c r="D2" s="12" t="s">
         <v>86</v>
       </c>
-      <c r="E2" s="13" t="s">
+      <c r="E2" s="12" t="s">
         <v>87</v>
       </c>
-      <c r="F2" s="13" t="s">
+      <c r="F2" s="12" t="s">
         <v>88</v>
       </c>
-      <c r="G2" s="13" t="s">
+      <c r="G2" s="12" t="s">
         <v>89</v>
       </c>
-      <c r="H2" s="13" t="s">
+      <c r="H2" s="12" t="s">
         <v>50</v>
       </c>
-      <c r="I2" s="14" t="n">
+      <c r="I2" s="13" t="n">
         <v>45</v>
       </c>
-      <c r="J2" s="14" t="n">
+      <c r="J2" s="13" t="n">
         <v>45</v>
       </c>
-      <c r="K2" s="15" t="n">
+      <c r="K2" s="14" t="n">
         <f aca="false">IF(I2="","",IFERROR(I2*INDEX(rates!$C$5:$C$12,MATCH($H2,rates!$A$5:$A$12,0)),"check currency code"))</f>
         <v>35100</v>
       </c>
-      <c r="L2" s="15" t="n">
+      <c r="L2" s="14" t="n">
         <f aca="false">IF(J2="","",IFERROR(J2*INDEX(rates!$C$5:$C$12,MATCH($H2,rates!$A$5:$A$12,0)),"check currency code"))</f>
         <v>35100</v>
       </c>
-      <c r="M2" s="13" t="n">
+      <c r="M2" s="12" t="n">
         <v>30</v>
       </c>
-      <c r="N2" s="13" t="n">
+      <c r="N2" s="12" t="n">
         <v>40</v>
       </c>
-      <c r="O2" s="13" t="n">
+      <c r="O2" s="12" t="n">
         <v>3</v>
       </c>
-      <c r="P2" s="13" t="s">
+      <c r="P2" s="12" t="s">
         <v>90</v>
       </c>
-      <c r="Q2" s="16" t="s">
+      <c r="Q2" s="15" t="s">
         <v>91</v>
       </c>
-      <c r="R2" s="16" t="s">
+      <c r="R2" s="15" t="s">
         <v>92</v>
       </c>
-      <c r="S2" s="13" t="s">
+      <c r="S2" s="12" t="s">
         <v>93</v>
       </c>
-      <c r="T2" s="13" t="s">
+      <c r="T2" s="12" t="s">
         <v>94</v>
       </c>
-      <c r="U2" s="13" t="n">
+      <c r="U2" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="V2" s="13" t="s">
+      <c r="V2" s="12" t="s">
         <v>95</v>
       </c>
-      <c r="W2" s="13" t="s">
+      <c r="W2" s="12" t="s">
         <v>96</v>
       </c>
-      <c r="X2" s="17" t="s">
+      <c r="X2" s="16" t="s">
         <v>97</v>
       </c>
-      <c r="Y2" s="18" t="s">
+      <c r="Y2" s="17" t="s">
         <v>98</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="19" t="s">
+      <c r="A3" s="18" t="s">
         <v>99</v>
       </c>
-      <c r="B3" s="19" t="s">
+      <c r="B3" s="18" t="s">
         <v>84</v>
       </c>
-      <c r="C3" s="19" t="s">
+      <c r="C3" s="18" t="s">
         <v>85</v>
       </c>
-      <c r="D3" s="19" t="s">
+      <c r="D3" s="18" t="s">
         <v>86</v>
       </c>
-      <c r="E3" s="19" t="s">
+      <c r="E3" s="18" t="s">
         <v>87</v>
       </c>
-      <c r="F3" s="19" t="s">
+      <c r="F3" s="18" t="s">
         <v>88</v>
       </c>
-      <c r="G3" s="19" t="s">
+      <c r="G3" s="18" t="s">
         <v>89</v>
       </c>
-      <c r="H3" s="19" t="s">
+      <c r="H3" s="18" t="s">
         <v>50</v>
       </c>
-      <c r="I3" s="14" t="n">
+      <c r="I3" s="13" t="n">
         <v>45</v>
       </c>
-      <c r="J3" s="14" t="n">
+      <c r="J3" s="13" t="n">
         <v>45</v>
       </c>
-      <c r="K3" s="20" t="n">
+      <c r="K3" s="19" t="n">
         <f aca="false">IF(I3="","",IFERROR(I3*INDEX(rates!$C$5:$C$12,MATCH($H3,rates!$A$5:$A$12,0)),"check currency code"))</f>
         <v>35100</v>
       </c>
-      <c r="L3" s="20" t="n">
+      <c r="L3" s="19" t="n">
         <f aca="false">IF(J3="","",IFERROR(J3*INDEX(rates!$C$5:$C$12,MATCH($H3,rates!$A$5:$A$12,0)),"check currency code"))</f>
         <v>35100</v>
       </c>
-      <c r="M3" s="13" t="n">
+      <c r="M3" s="12" t="n">
         <v>30</v>
       </c>
-      <c r="N3" s="13" t="n">
+      <c r="N3" s="12" t="n">
         <v>40</v>
       </c>
-      <c r="O3" s="13" t="n">
+      <c r="O3" s="12" t="n">
         <v>3</v>
       </c>
-      <c r="P3" s="13" t="s">
+      <c r="P3" s="12" t="s">
         <v>90</v>
       </c>
-      <c r="Q3" s="21" t="s">
+      <c r="Q3" s="20" t="s">
         <v>91</v>
       </c>
-      <c r="R3" s="21" t="s">
+      <c r="R3" s="20" t="s">
         <v>92</v>
       </c>
-      <c r="S3" s="13" t="s">
+      <c r="S3" s="12" t="s">
         <v>93</v>
       </c>
-      <c r="T3" s="13" t="s">
+      <c r="T3" s="12" t="s">
         <v>94</v>
       </c>
-      <c r="U3" s="22" t="n">
+      <c r="U3" s="21" t="n">
         <v>2</v>
       </c>
-      <c r="V3" s="13" t="s">
+      <c r="V3" s="12" t="s">
         <v>95</v>
       </c>
-      <c r="W3" s="22" t="s">
+      <c r="W3" s="21" t="s">
         <v>100</v>
       </c>
-      <c r="X3" s="23" t="s">
+      <c r="X3" s="22" t="s">
         <v>97</v>
       </c>
-      <c r="Y3" s="18" t="s">
+      <c r="Y3" s="17" t="s">
         <v>98</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="19" t="s">
+      <c r="A4" s="18" t="s">
         <v>101</v>
       </c>
-      <c r="B4" s="19" t="s">
+      <c r="B4" s="18" t="s">
         <v>84</v>
       </c>
-      <c r="C4" s="19" t="s">
+      <c r="C4" s="18" t="s">
         <v>85</v>
       </c>
-      <c r="D4" s="19" t="s">
+      <c r="D4" s="18" t="s">
         <v>86</v>
       </c>
-      <c r="E4" s="19" t="s">
+      <c r="E4" s="18" t="s">
         <v>102</v>
       </c>
-      <c r="F4" s="19" t="s">
+      <c r="F4" s="18" t="s">
         <v>103</v>
       </c>
-      <c r="G4" s="19" t="s">
+      <c r="G4" s="18" t="s">
         <v>104</v>
       </c>
-      <c r="H4" s="19" t="s">
+      <c r="H4" s="18" t="s">
         <v>50</v>
       </c>
-      <c r="I4" s="24" t="n">
+      <c r="I4" s="23" t="n">
         <v>60</v>
       </c>
-      <c r="J4" s="24" t="n">
+      <c r="J4" s="23" t="n">
         <v>60</v>
       </c>
-      <c r="K4" s="20" t="n">
+      <c r="K4" s="19" t="n">
         <f aca="false">IF(I4="","",IFERROR(I4*INDEX(rates!$C$5:$C$12,MATCH($H4,rates!$A$5:$A$12,0)),"check currency code"))</f>
         <v>46800</v>
       </c>
-      <c r="L4" s="20" t="n">
+      <c r="L4" s="19" t="n">
         <f aca="false">IF(J4="","",IFERROR(J4*INDEX(rates!$C$5:$C$12,MATCH($H4,rates!$A$5:$A$12,0)),"check currency code"))</f>
         <v>46800</v>
       </c>
-      <c r="M4" s="22" t="n">
+      <c r="M4" s="21" t="n">
         <v>60</v>
       </c>
-      <c r="N4" s="22" t="n">
+      <c r="N4" s="21" t="n">
         <v>90</v>
       </c>
-      <c r="O4" s="25" t="n">
+      <c r="O4" s="24" t="n">
         <v>1</v>
       </c>
-      <c r="P4" s="26" t="s">
+      <c r="P4" s="25" t="s">
         <v>90</v>
       </c>
-      <c r="Q4" s="21" t="s">
+      <c r="Q4" s="20" t="s">
         <v>91</v>
       </c>
-      <c r="R4" s="21" t="s">
+      <c r="R4" s="20" t="s">
         <v>105</v>
       </c>
-      <c r="S4" s="22" t="s">
+      <c r="S4" s="21" t="s">
         <v>106</v>
       </c>
-      <c r="T4" s="25" t="s">
+      <c r="T4" s="24" t="s">
         <v>94</v>
       </c>
-      <c r="U4" s="27" t="n">
+      <c r="U4" s="26" t="n">
         <v>2</v>
       </c>
-      <c r="V4" s="22" t="s">
+      <c r="V4" s="21" t="s">
         <v>107</v>
       </c>
-      <c r="W4" s="22" t="s">
+      <c r="W4" s="21" t="s">
         <v>108</v>
       </c>
-      <c r="X4" s="23" t="s">
+      <c r="X4" s="22" t="s">
         <v>97</v>
       </c>
-      <c r="Y4" s="18" t="s">
+      <c r="Y4" s="17" t="s">
         <v>98</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="19" t="s">
+      <c r="A5" s="18" t="s">
         <v>109</v>
       </c>
-      <c r="B5" s="19" t="s">
+      <c r="B5" s="18" t="s">
         <v>84</v>
       </c>
-      <c r="C5" s="19" t="s">
+      <c r="C5" s="18" t="s">
         <v>85</v>
       </c>
-      <c r="D5" s="19" t="s">
+      <c r="D5" s="18" t="s">
         <v>86</v>
       </c>
-      <c r="E5" s="19" t="s">
+      <c r="E5" s="18" t="s">
         <v>87</v>
       </c>
-      <c r="F5" s="19" t="s">
+      <c r="F5" s="18" t="s">
         <v>110</v>
       </c>
-      <c r="G5" s="19" t="s">
+      <c r="G5" s="18" t="s">
         <v>111</v>
       </c>
-      <c r="H5" s="19" t="s">
+      <c r="H5" s="18" t="s">
         <v>50</v>
       </c>
-      <c r="I5" s="24" t="n">
+      <c r="I5" s="23" t="n">
         <v>400</v>
       </c>
-      <c r="J5" s="24" t="n">
+      <c r="J5" s="23" t="n">
         <v>600</v>
       </c>
-      <c r="K5" s="20" t="n">
+      <c r="K5" s="19" t="n">
         <f aca="false">IF(I5="","",IFERROR(I5*INDEX(rates!$C$5:$C$12,MATCH($H5,rates!$A$5:$A$12,0)),"check currency code"))</f>
         <v>312000</v>
       </c>
-      <c r="L5" s="20" t="n">
+      <c r="L5" s="19" t="n">
         <f aca="false">IF(J5="","",IFERROR(J5*INDEX(rates!$C$5:$C$12,MATCH($H5,rates!$A$5:$A$12,0)),"check currency code"))</f>
         <v>468000</v>
       </c>
-      <c r="M5" s="25" t="n">
+      <c r="M5" s="24" t="n">
         <v>45</v>
       </c>
-      <c r="N5" s="25" t="n">
+      <c r="N5" s="24" t="n">
         <v>60</v>
       </c>
-      <c r="O5" s="25" t="n">
+      <c r="O5" s="24" t="n">
         <v>4</v>
       </c>
-      <c r="P5" s="26" t="s">
+      <c r="P5" s="25" t="s">
         <v>112</v>
       </c>
-      <c r="Q5" s="21" t="s">
+      <c r="Q5" s="20" t="s">
         <v>113</v>
       </c>
-      <c r="R5" s="21" t="s">
+      <c r="R5" s="20" t="s">
         <v>92</v>
       </c>
-      <c r="S5" s="22" t="s">
+      <c r="S5" s="21" t="s">
         <v>114</v>
       </c>
-      <c r="T5" s="13" t="s">
+      <c r="T5" s="12" t="s">
         <v>94</v>
       </c>
-      <c r="U5" s="22" t="n">
+      <c r="U5" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="V5" s="22" t="s">
+      <c r="V5" s="21" t="s">
         <v>115</v>
       </c>
-      <c r="W5" s="22" t="s">
+      <c r="W5" s="21" t="s">
         <v>116</v>
       </c>
-      <c r="X5" s="23" t="s">
+      <c r="X5" s="22" t="s">
         <v>97</v>
       </c>
-      <c r="Y5" s="18" t="s">
+      <c r="Y5" s="17" t="s">
         <v>117</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="46.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="19" t="s">
+      <c r="A6" s="18" t="s">
         <v>118</v>
       </c>
-      <c r="B6" s="19" t="s">
+      <c r="B6" s="18" t="s">
         <v>84</v>
       </c>
-      <c r="C6" s="19" t="s">
+      <c r="C6" s="18" t="s">
         <v>85</v>
       </c>
-      <c r="D6" s="19" t="s">
+      <c r="D6" s="18" t="s">
         <v>86</v>
       </c>
-      <c r="E6" s="19" t="s">
+      <c r="E6" s="18" t="s">
         <v>87</v>
       </c>
-      <c r="F6" s="19" t="s">
+      <c r="F6" s="18" t="s">
         <v>119</v>
       </c>
-      <c r="G6" s="19" t="s">
+      <c r="G6" s="18" t="s">
         <v>120</v>
       </c>
-      <c r="H6" s="19" t="s">
+      <c r="H6" s="18" t="s">
         <v>50</v>
       </c>
-      <c r="I6" s="24" t="n">
+      <c r="I6" s="23" t="n">
         <v>450</v>
       </c>
-      <c r="J6" s="24" t="n">
+      <c r="J6" s="23" t="n">
         <v>700</v>
       </c>
-      <c r="K6" s="20" t="n">
+      <c r="K6" s="19" t="n">
         <f aca="false">IF(I6="","",IFERROR(I6*INDEX(rates!$C$5:$C$12,MATCH($H6,rates!$A$5:$A$12,0)),"check currency code"))</f>
         <v>351000</v>
       </c>
-      <c r="L6" s="20" t="n">
+      <c r="L6" s="19" t="n">
         <f aca="false">IF(J6="","",IFERROR(J6*INDEX(rates!$C$5:$C$12,MATCH($H6,rates!$A$5:$A$12,0)),"check currency code"))</f>
         <v>546000</v>
       </c>
-      <c r="M6" s="25" t="n">
+      <c r="M6" s="24" t="n">
         <v>45</v>
       </c>
-      <c r="N6" s="25" t="n">
+      <c r="N6" s="24" t="n">
         <v>60</v>
       </c>
-      <c r="O6" s="25" t="n">
+      <c r="O6" s="24" t="n">
         <v>4</v>
       </c>
-      <c r="P6" s="26" t="s">
+      <c r="P6" s="25" t="s">
         <v>112</v>
       </c>
-      <c r="Q6" s="21" t="s">
+      <c r="Q6" s="20" t="s">
         <v>113</v>
       </c>
-      <c r="R6" s="21" t="s">
+      <c r="R6" s="20" t="s">
         <v>92</v>
       </c>
-      <c r="S6" s="28" t="s">
+      <c r="S6" s="21" t="s">
         <v>121</v>
       </c>
-      <c r="T6" s="22" t="s">
+      <c r="T6" s="21" t="s">
         <v>120</v>
       </c>
-      <c r="U6" s="22" t="n">
+      <c r="U6" s="21" t="n">
         <v>1</v>
       </c>
-      <c r="V6" s="28" t="s">
+      <c r="V6" s="21" t="s">
         <v>122</v>
       </c>
-      <c r="W6" s="28" t="s">
+      <c r="W6" s="21" t="s">
         <v>123</v>
       </c>
-      <c r="X6" s="23" t="s">
+      <c r="X6" s="22" t="s">
         <v>97</v>
       </c>
-      <c r="Y6" s="18" t="s">
+      <c r="Y6" s="17" t="s">
         <v>117</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="19" t="s">
+      <c r="A7" s="18" t="s">
         <v>124</v>
       </c>
-      <c r="B7" s="19" t="s">
+      <c r="B7" s="18" t="s">
         <v>84</v>
       </c>
-      <c r="C7" s="19" t="s">
+      <c r="C7" s="18" t="s">
         <v>85</v>
       </c>
-      <c r="D7" s="19" t="s">
+      <c r="D7" s="18" t="s">
         <v>86</v>
       </c>
-      <c r="E7" s="19" t="s">
+      <c r="E7" s="18" t="s">
         <v>87</v>
       </c>
-      <c r="F7" s="19" t="s">
+      <c r="F7" s="18" t="s">
         <v>125</v>
       </c>
-      <c r="G7" s="19" t="s">
+      <c r="G7" s="18" t="s">
         <v>126</v>
       </c>
-      <c r="H7" s="19" t="s">
+      <c r="H7" s="18" t="s">
         <v>50</v>
       </c>
-      <c r="I7" s="24" t="n">
+      <c r="I7" s="23" t="n">
         <v>800</v>
       </c>
-      <c r="J7" s="24" t="n">
+      <c r="J7" s="23" t="n">
         <v>1200</v>
       </c>
-      <c r="K7" s="20" t="n">
+      <c r="K7" s="19" t="n">
         <f aca="false">IF(I7="","",IFERROR(I7*INDEX(rates!$C$5:$C$12,MATCH($H7,rates!$A$5:$A$12,0)),"check currency code"))</f>
         <v>624000</v>
       </c>
-      <c r="L7" s="20" t="n">
+      <c r="L7" s="19" t="n">
         <f aca="false">IF(J7="","",IFERROR(J7*INDEX(rates!$C$5:$C$12,MATCH($H7,rates!$A$5:$A$12,0)),"check currency code"))</f>
         <v>936000</v>
       </c>
-      <c r="M7" s="22" t="n">
+      <c r="M7" s="21" t="n">
         <v>45</v>
       </c>
-      <c r="N7" s="22" t="n">
+      <c r="N7" s="21" t="n">
         <v>60</v>
       </c>
-      <c r="O7" s="25" t="n">
+      <c r="O7" s="24" t="n">
         <v>5</v>
       </c>
-      <c r="P7" s="26" t="s">
+      <c r="P7" s="25" t="s">
         <v>112</v>
       </c>
-      <c r="Q7" s="21" t="s">
+      <c r="Q7" s="20" t="s">
         <v>113</v>
       </c>
-      <c r="R7" s="21" t="s">
+      <c r="R7" s="20" t="s">
         <v>92</v>
       </c>
-      <c r="S7" s="28" t="s">
+      <c r="S7" s="21" t="s">
         <v>127</v>
       </c>
-      <c r="T7" s="22" t="s">
+      <c r="T7" s="21" t="s">
         <v>94</v>
       </c>
-      <c r="U7" s="22" t="n">
+      <c r="U7" s="21" t="n">
         <v>1</v>
       </c>
-      <c r="V7" s="28" t="s">
+      <c r="V7" s="21" t="s">
         <v>128</v>
       </c>
-      <c r="W7" s="28" t="s">
+      <c r="W7" s="21" t="s">
         <v>129</v>
       </c>
-      <c r="X7" s="23" t="s">
+      <c r="X7" s="22" t="s">
         <v>97</v>
       </c>
-      <c r="Y7" s="18" t="s">
+      <c r="Y7" s="17" t="s">
         <v>117</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="67.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="19" t="s">
+      <c r="A8" s="18" t="s">
         <v>130</v>
       </c>
-      <c r="B8" s="19" t="s">
+      <c r="B8" s="18" t="s">
         <v>84</v>
       </c>
-      <c r="C8" s="19" t="s">
+      <c r="C8" s="18" t="s">
         <v>85</v>
       </c>
-      <c r="D8" s="19" t="s">
+      <c r="D8" s="18" t="s">
         <v>131</v>
       </c>
-      <c r="E8" s="19" t="s">
+      <c r="E8" s="18" t="s">
         <v>132</v>
       </c>
-      <c r="F8" s="19" t="s">
+      <c r="F8" s="18" t="s">
         <v>103</v>
       </c>
-      <c r="G8" s="19" t="s">
+      <c r="G8" s="18" t="s">
         <v>133</v>
       </c>
-      <c r="H8" s="19" t="s">
+      <c r="H8" s="18" t="s">
         <v>50</v>
       </c>
-      <c r="I8" s="24" t="n">
+      <c r="I8" s="23" t="n">
         <v>30</v>
       </c>
-      <c r="J8" s="24" t="n">
+      <c r="J8" s="23" t="n">
         <v>30</v>
       </c>
-      <c r="K8" s="20" t="n">
+      <c r="K8" s="19" t="n">
         <f aca="false">IF(I8="","",IFERROR(I8*INDEX(rates!$C$5:$C$12,MATCH($H8,rates!$A$5:$A$12,0)),"check currency code"))</f>
         <v>23400</v>
       </c>
-      <c r="L8" s="20" t="n">
+      <c r="L8" s="19" t="n">
         <f aca="false">IF(J8="","",IFERROR(J8*INDEX(rates!$C$5:$C$12,MATCH($H8,rates!$A$5:$A$12,0)),"check currency code"))</f>
         <v>23400</v>
       </c>
-      <c r="M8" s="28" t="n">
+      <c r="M8" s="21" t="n">
         <v>23</v>
       </c>
-      <c r="N8" s="28" t="n">
+      <c r="N8" s="21" t="n">
         <v>45</v>
       </c>
-      <c r="O8" s="28" t="n">
+      <c r="O8" s="21" t="n">
         <v>2</v>
       </c>
-      <c r="P8" s="26" t="s">
+      <c r="P8" s="25" t="s">
         <v>90</v>
       </c>
-      <c r="Q8" s="21" t="s">
+      <c r="Q8" s="20" t="s">
         <v>134</v>
       </c>
-      <c r="R8" s="21" t="s">
+      <c r="R8" s="20" t="s">
         <v>92</v>
       </c>
-      <c r="S8" s="28" t="s">
+      <c r="S8" s="21" t="s">
         <v>135</v>
       </c>
-      <c r="T8" s="13" t="s">
+      <c r="T8" s="12" t="s">
         <v>94</v>
       </c>
-      <c r="U8" s="28" t="n">
+      <c r="U8" s="21" t="n">
         <v>3</v>
       </c>
-      <c r="V8" s="28" t="s">
+      <c r="V8" s="21" t="s">
         <v>136</v>
       </c>
-      <c r="W8" s="28" t="s">
+      <c r="W8" s="21" t="s">
         <v>137</v>
       </c>
-      <c r="X8" s="23" t="s">
+      <c r="X8" s="22" t="s">
         <v>97</v>
       </c>
-      <c r="Y8" s="18" t="s">
+      <c r="Y8" s="17" t="s">
         <v>98</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="58.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="19" t="s">
+      <c r="A9" s="18" t="s">
         <v>138</v>
       </c>
-      <c r="B9" s="19" t="s">
+      <c r="B9" s="18" t="s">
         <v>84</v>
       </c>
-      <c r="C9" s="19" t="s">
+      <c r="C9" s="18" t="s">
         <v>85</v>
       </c>
-      <c r="D9" s="19" t="s">
+      <c r="D9" s="18" t="s">
         <v>131</v>
       </c>
-      <c r="E9" s="19" t="s">
+      <c r="E9" s="18" t="s">
         <v>139</v>
       </c>
-      <c r="F9" s="19" t="s">
+      <c r="F9" s="18" t="s">
         <v>88</v>
       </c>
-      <c r="G9" s="19" t="s">
+      <c r="G9" s="18" t="s">
         <v>140</v>
       </c>
-      <c r="H9" s="19" t="s">
+      <c r="H9" s="18" t="s">
         <v>50</v>
       </c>
-      <c r="I9" s="29" t="n">
+      <c r="I9" s="27" t="n">
         <v>33</v>
       </c>
-      <c r="J9" s="29" t="n">
+      <c r="J9" s="27" t="n">
         <v>33</v>
       </c>
-      <c r="K9" s="20" t="n">
+      <c r="K9" s="19" t="n">
         <f aca="false">IF(I9="","",IFERROR(I9*INDEX(rates!$C$5:$C$12,MATCH($H9,rates!$A$5:$A$12,0)),"check currency code"))</f>
         <v>25740</v>
       </c>
-      <c r="L9" s="20" t="n">
+      <c r="L9" s="19" t="n">
         <f aca="false">IF(J9="","",IFERROR(J9*INDEX(rates!$C$5:$C$12,MATCH($H9,rates!$A$5:$A$12,0)),"check currency code"))</f>
         <v>25740</v>
       </c>
-      <c r="M9" s="28" t="n">
+      <c r="M9" s="21" t="n">
         <v>17</v>
       </c>
-      <c r="N9" s="28" t="n">
+      <c r="N9" s="21" t="n">
         <v>20</v>
       </c>
-      <c r="O9" s="28" t="n">
+      <c r="O9" s="21" t="n">
         <v>3</v>
       </c>
-      <c r="P9" s="26" t="s">
+      <c r="P9" s="25" t="s">
         <v>90</v>
       </c>
-      <c r="Q9" s="21" t="s">
+      <c r="Q9" s="20" t="s">
         <v>141</v>
       </c>
-      <c r="R9" s="21" t="s">
+      <c r="R9" s="20" t="s">
         <v>92</v>
       </c>
-      <c r="S9" s="28" t="s">
+      <c r="S9" s="21" t="s">
         <v>142</v>
       </c>
-      <c r="T9" s="13" t="s">
+      <c r="T9" s="12" t="s">
         <v>94</v>
       </c>
-      <c r="U9" s="28" t="n">
+      <c r="U9" s="21" t="n">
         <v>2</v>
       </c>
-      <c r="V9" s="28" t="s">
+      <c r="V9" s="21" t="s">
         <v>143</v>
       </c>
-      <c r="W9" s="28" t="s">
+      <c r="W9" s="21" t="s">
         <v>144</v>
       </c>
-      <c r="X9" s="23" t="s">
+      <c r="X9" s="22" t="s">
         <v>97</v>
       </c>
-      <c r="Y9" s="18" t="s">
+      <c r="Y9" s="17" t="s">
         <v>98</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="19" t="s">
+      <c r="A10" s="18" t="s">
         <v>145</v>
       </c>
-      <c r="B10" s="19" t="s">
+      <c r="B10" s="18" t="s">
         <v>84</v>
       </c>
-      <c r="C10" s="19" t="s">
+      <c r="C10" s="18" t="s">
         <v>85</v>
       </c>
-      <c r="D10" s="19" t="s">
+      <c r="D10" s="18" t="s">
         <v>131</v>
       </c>
-      <c r="E10" s="19" t="s">
+      <c r="E10" s="18" t="s">
         <v>102</v>
       </c>
-      <c r="F10" s="19" t="s">
+      <c r="F10" s="18" t="s">
         <v>110</v>
       </c>
-      <c r="G10" s="19" t="s">
+      <c r="G10" s="18" t="s">
         <v>111</v>
       </c>
-      <c r="H10" s="19" t="s">
+      <c r="H10" s="18" t="s">
         <v>50</v>
       </c>
-      <c r="I10" s="24" t="n">
+      <c r="I10" s="23" t="n">
         <v>400</v>
       </c>
-      <c r="J10" s="24" t="n">
+      <c r="J10" s="23" t="n">
         <v>500</v>
       </c>
-      <c r="K10" s="20" t="n">
+      <c r="K10" s="19" t="n">
         <f aca="false">IF(I10="","",IFERROR(I10*INDEX(rates!$C$5:$C$12,MATCH($H10,rates!$A$5:$A$12,0)),"check currency code"))</f>
         <v>312000</v>
       </c>
-      <c r="L10" s="20" t="n">
+      <c r="L10" s="19" t="n">
         <f aca="false">IF(J10="","",IFERROR(J10*INDEX(rates!$C$5:$C$12,MATCH($H10,rates!$A$5:$A$12,0)),"check currency code"))</f>
         <v>390000</v>
       </c>
-      <c r="M10" s="25" t="n">
+      <c r="M10" s="24" t="n">
         <v>20</v>
       </c>
-      <c r="N10" s="25" t="n">
+      <c r="N10" s="24" t="n">
         <v>30</v>
       </c>
-      <c r="O10" s="28" t="n">
+      <c r="O10" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="P10" s="26" t="s">
+      <c r="P10" s="25" t="s">
         <v>112</v>
       </c>
-      <c r="Q10" s="21" t="s">
+      <c r="Q10" s="20" t="s">
         <v>113</v>
       </c>
-      <c r="R10" s="21" t="s">
+      <c r="R10" s="20" t="s">
         <v>92</v>
       </c>
-      <c r="S10" s="28" t="s">
+      <c r="S10" s="21" t="s">
         <v>146</v>
       </c>
-      <c r="T10" s="13" t="s">
+      <c r="T10" s="12" t="s">
         <v>94</v>
       </c>
-      <c r="U10" s="25" t="n">
+      <c r="U10" s="24" t="n">
         <v>4</v>
       </c>
-      <c r="V10" s="28" t="s">
+      <c r="V10" s="21" t="s">
         <v>147</v>
       </c>
-      <c r="W10" s="25" t="s">
+      <c r="W10" s="24" t="s">
         <v>148</v>
       </c>
-      <c r="X10" s="23" t="s">
+      <c r="X10" s="22" t="s">
         <v>97</v>
       </c>
-      <c r="Y10" s="18" t="s">
+      <c r="Y10" s="17" t="s">
         <v>117</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="19" t="s">
+      <c r="A11" s="18" t="s">
         <v>149</v>
       </c>
-      <c r="B11" s="19" t="s">
+      <c r="B11" s="18" t="s">
         <v>150</v>
       </c>
-      <c r="C11" s="19" t="s">
+      <c r="C11" s="18" t="s">
         <v>151</v>
       </c>
-      <c r="D11" s="19" t="s">
+      <c r="D11" s="18" t="s">
         <v>152</v>
       </c>
-      <c r="E11" s="19" t="s">
+      <c r="E11" s="18" t="s">
         <v>153</v>
       </c>
-      <c r="F11" s="19" t="s">
+      <c r="F11" s="18" t="s">
         <v>88</v>
       </c>
-      <c r="G11" s="19" t="s">
+      <c r="G11" s="18" t="s">
         <v>154</v>
       </c>
-      <c r="H11" s="19" t="s">
+      <c r="H11" s="18" t="s">
         <v>52</v>
       </c>
-      <c r="I11" s="29" t="n">
+      <c r="I11" s="27" t="n">
         <v>11500</v>
       </c>
-      <c r="J11" s="29" t="n">
+      <c r="J11" s="27" t="n">
         <v>13000</v>
       </c>
-      <c r="K11" s="30" t="n">
+      <c r="K11" s="19" t="n">
         <f aca="false">IF(I11="","",IFERROR(I11*INDEX(rates!$C$5:$C$12,MATCH($H11,rates!$A$5:$A$12,0)),"check currency code"))</f>
         <v>218500</v>
       </c>
-      <c r="L11" s="20" t="n">
+      <c r="L11" s="19" t="n">
         <f aca="false">IF(J11="","",IFERROR(J11*INDEX(rates!$C$5:$C$12,MATCH($H11,rates!$A$5:$A$12,0)),"check currency code"))</f>
         <v>247000</v>
       </c>
-      <c r="M11" s="25" t="n">
+      <c r="M11" s="24" t="n">
         <v>43</v>
       </c>
-      <c r="N11" s="25" t="n">
+      <c r="N11" s="24" t="n">
         <v>51</v>
       </c>
       <c r="O11" s="28" t="n">
         <v>4</v>
       </c>
-      <c r="P11" s="28" t="s">
+      <c r="P11" s="21" t="s">
         <v>112</v>
       </c>
-      <c r="Q11" s="23" t="s">
+      <c r="Q11" s="22" t="s">
         <v>155</v>
       </c>
-      <c r="R11" s="23" t="s">
+      <c r="R11" s="22" t="s">
         <v>156</v>
       </c>
-      <c r="S11" s="31" t="s">
+      <c r="S11" s="29" t="s">
         <v>157</v>
       </c>
-      <c r="T11" s="28" t="s">
+      <c r="T11" s="21" t="s">
         <v>94</v>
       </c>
-      <c r="U11" s="28" t="n">
+      <c r="U11" s="21" t="n">
         <v>2</v>
       </c>
-      <c r="V11" s="28" t="s">
+      <c r="V11" s="21" t="s">
         <v>158</v>
       </c>
-      <c r="W11" s="31" t="s">
+      <c r="W11" s="29" t="s">
         <v>159</v>
       </c>
-      <c r="X11" s="23" t="s">
+      <c r="X11" s="22" t="s">
         <v>97</v>
       </c>
-      <c r="Y11" s="18" t="s">
+      <c r="Y11" s="17" t="s">
         <v>98</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="91.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="19" t="s">
+      <c r="A12" s="18" t="s">
         <v>160</v>
       </c>
-      <c r="B12" s="19" t="s">
+      <c r="B12" s="18" t="s">
         <v>150</v>
       </c>
-      <c r="C12" s="19" t="s">
+      <c r="C12" s="18" t="s">
         <v>151</v>
       </c>
-      <c r="D12" s="19" t="s">
+      <c r="D12" s="18" t="s">
         <v>152</v>
       </c>
-      <c r="E12" s="19" t="s">
+      <c r="E12" s="18" t="s">
         <v>161</v>
       </c>
-      <c r="F12" s="19" t="s">
+      <c r="F12" s="18" t="s">
         <v>88</v>
       </c>
-      <c r="G12" s="19" t="s">
+      <c r="G12" s="18" t="s">
         <v>162</v>
       </c>
-      <c r="H12" s="19" t="s">
+      <c r="H12" s="18" t="s">
         <v>52</v>
       </c>
-      <c r="I12" s="24" t="n">
+      <c r="I12" s="23" t="n">
         <v>4150</v>
       </c>
-      <c r="J12" s="24" t="n">
+      <c r="J12" s="23" t="n">
         <v>4150</v>
       </c>
-      <c r="K12" s="20" t="n">
+      <c r="K12" s="19" t="n">
         <f aca="false">IF(I12="","",IFERROR(I12*INDEX(rates!$C$5:$C$12,MATCH($H12,rates!$A$5:$A$12,0)),"check currency code"))</f>
         <v>78850</v>
       </c>
-      <c r="L12" s="20" t="n">
+      <c r="L12" s="19" t="n">
         <f aca="false">IF(J12="","",IFERROR(J12*INDEX(rates!$C$5:$C$12,MATCH($H12,rates!$A$5:$A$12,0)),"check currency code"))</f>
         <v>78850</v>
       </c>
-      <c r="M12" s="25" t="n">
+      <c r="M12" s="24" t="n">
         <v>59</v>
       </c>
-      <c r="N12" s="25" t="n">
+      <c r="N12" s="24" t="n">
         <v>66</v>
       </c>
-      <c r="O12" s="28" t="n">
+      <c r="O12" s="21" t="n">
         <v>2</v>
       </c>
-      <c r="P12" s="28" t="s">
+      <c r="P12" s="21" t="s">
         <v>90</v>
       </c>
-      <c r="Q12" s="23" t="s">
+      <c r="Q12" s="22" t="s">
         <v>163</v>
       </c>
-      <c r="R12" s="23" t="s">
+      <c r="R12" s="22" t="s">
         <v>164</v>
       </c>
-      <c r="S12" s="32" t="s">
+      <c r="S12" s="30" t="s">
         <v>165</v>
       </c>
-      <c r="T12" s="28" t="s">
+      <c r="T12" s="21" t="s">
         <v>94</v>
       </c>
-      <c r="U12" s="28" t="n">
+      <c r="U12" s="21" t="n">
         <v>2</v>
       </c>
-      <c r="V12" s="28" t="s">
+      <c r="V12" s="21" t="s">
         <v>166</v>
       </c>
-      <c r="W12" s="33" t="s">
+      <c r="W12" s="31" t="s">
         <v>167</v>
       </c>
-      <c r="X12" s="23" t="s">
+      <c r="X12" s="22" t="s">
         <v>97</v>
       </c>
-      <c r="Y12" s="18" t="s">
+      <c r="Y12" s="17" t="s">
         <v>98</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="121.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="19" t="s">
+      <c r="A13" s="18" t="s">
         <v>168</v>
       </c>
-      <c r="B13" s="19" t="s">
+      <c r="B13" s="18" t="s">
         <v>150</v>
       </c>
-      <c r="C13" s="19" t="s">
+      <c r="C13" s="18" t="s">
         <v>151</v>
       </c>
-      <c r="D13" s="19" t="s">
+      <c r="D13" s="18" t="s">
         <v>152</v>
       </c>
-      <c r="E13" s="19" t="s">
+      <c r="E13" s="18" t="s">
         <v>169</v>
       </c>
-      <c r="F13" s="19" t="s">
+      <c r="F13" s="18" t="s">
         <v>103</v>
       </c>
-      <c r="G13" s="19" t="s">
+      <c r="G13" s="18" t="s">
         <v>170</v>
       </c>
-      <c r="H13" s="19" t="s">
+      <c r="H13" s="18" t="s">
         <v>52</v>
       </c>
-      <c r="I13" s="29" t="n">
+      <c r="I13" s="27" t="n">
         <v>17000</v>
       </c>
-      <c r="J13" s="29" t="n">
+      <c r="J13" s="27" t="n">
         <v>17000</v>
       </c>
-      <c r="K13" s="20" t="n">
+      <c r="K13" s="19" t="n">
         <f aca="false">IF(I13="","",IFERROR(I13*INDEX(rates!$C$5:$C$12,MATCH($H13,rates!$A$5:$A$12,0)),"check currency code"))</f>
         <v>323000</v>
       </c>
-      <c r="L13" s="20" t="n">
+      <c r="L13" s="19" t="n">
         <f aca="false">IF(J13="","",IFERROR(J13*INDEX(rates!$C$5:$C$12,MATCH($H13,rates!$A$5:$A$12,0)),"check currency code"))</f>
         <v>323000</v>
       </c>
-      <c r="M13" s="25" t="n">
+      <c r="M13" s="24" t="n">
         <v>60</v>
       </c>
-      <c r="N13" s="25" t="n">
+      <c r="N13" s="24" t="n">
         <v>90</v>
       </c>
       <c r="O13" s="28" t="n">
         <v>4</v>
       </c>
-      <c r="P13" s="28" t="s">
+      <c r="P13" s="21" t="s">
         <v>112</v>
       </c>
-      <c r="Q13" s="23" t="s">
+      <c r="Q13" s="22" t="s">
         <v>163</v>
       </c>
-      <c r="R13" s="23" t="s">
+      <c r="R13" s="22" t="s">
         <v>171</v>
       </c>
-      <c r="S13" s="28" t="s">
+      <c r="S13" s="21" t="s">
         <v>172</v>
       </c>
-      <c r="T13" s="28" t="s">
+      <c r="T13" s="21" t="s">
         <v>94</v>
       </c>
-      <c r="U13" s="28" t="n">
+      <c r="U13" s="21" t="n">
         <v>2</v>
       </c>
-      <c r="V13" s="28" t="s">
+      <c r="V13" s="21" t="s">
         <v>173</v>
       </c>
-      <c r="W13" s="34" t="s">
+      <c r="W13" s="32" t="s">
         <v>174</v>
       </c>
-      <c r="X13" s="23" t="s">
+      <c r="X13" s="22" t="s">
         <v>97</v>
       </c>
-      <c r="Y13" s="18" t="s">
+      <c r="Y13" s="17" t="s">
         <v>98</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="19" t="s">
+      <c r="A14" s="18" t="s">
         <v>175</v>
       </c>
-      <c r="B14" s="19" t="s">
+      <c r="B14" s="18" t="s">
         <v>150</v>
       </c>
-      <c r="C14" s="19" t="s">
+      <c r="C14" s="18" t="s">
         <v>151</v>
       </c>
-      <c r="D14" s="19" t="s">
+      <c r="D14" s="18" t="s">
         <v>152</v>
       </c>
-      <c r="E14" s="19" t="s">
+      <c r="E14" s="18" t="s">
         <v>169</v>
       </c>
-      <c r="F14" s="19" t="s">
+      <c r="F14" s="18" t="s">
         <v>110</v>
       </c>
-      <c r="G14" s="19" t="s">
+      <c r="G14" s="18" t="s">
         <v>176</v>
       </c>
-      <c r="H14" s="19" t="s">
+      <c r="H14" s="18" t="s">
         <v>52</v>
       </c>
-      <c r="I14" s="24" t="n">
+      <c r="I14" s="23" t="n">
         <v>60000</v>
       </c>
-      <c r="J14" s="24" t="n">
+      <c r="J14" s="23" t="n">
         <v>100000</v>
       </c>
-      <c r="K14" s="20" t="n">
+      <c r="K14" s="19" t="n">
         <f aca="false">IF(I14="","",IFERROR(I14*INDEX(rates!$C$5:$C$12,MATCH($H14,rates!$A$5:$A$12,0)),"check currency code"))</f>
         <v>1140000</v>
       </c>
-      <c r="L14" s="20" t="n">
+      <c r="L14" s="19" t="n">
         <f aca="false">IF(J14="","",IFERROR(J14*INDEX(rates!$C$5:$C$12,MATCH($H14,rates!$A$5:$A$12,0)),"check currency code"))</f>
         <v>1900000</v>
       </c>
-      <c r="M14" s="25" t="n">
+      <c r="M14" s="24" t="n">
         <v>60</v>
       </c>
-      <c r="N14" s="25" t="n">
+      <c r="N14" s="24" t="n">
         <v>80</v>
       </c>
-      <c r="O14" s="25" t="n">
+      <c r="O14" s="24" t="n">
         <v>4</v>
       </c>
-      <c r="P14" s="26" t="s">
+      <c r="P14" s="25" t="s">
         <v>112</v>
       </c>
-      <c r="Q14" s="23" t="s">
+      <c r="Q14" s="22" t="s">
         <v>113</v>
       </c>
-      <c r="R14" s="21" t="s">
+      <c r="R14" s="20" t="s">
         <v>92</v>
       </c>
-      <c r="S14" s="28" t="s">
+      <c r="S14" s="21" t="s">
         <v>177</v>
       </c>
-      <c r="T14" s="28" t="s">
+      <c r="T14" s="21" t="s">
         <v>94</v>
       </c>
-      <c r="U14" s="25" t="n">
-        <v>4</v>
-      </c>
-      <c r="V14" s="28" t="s">
+      <c r="U14" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="V14" s="21" t="s">
         <v>178</v>
       </c>
-      <c r="W14" s="31" t="s">
+      <c r="W14" s="29" t="s">
         <v>179</v>
       </c>
-      <c r="X14" s="23" t="s">
+      <c r="X14" s="22" t="s">
         <v>97</v>
       </c>
-      <c r="Y14" s="18" t="s">
+      <c r="Y14" s="17" t="s">
         <v>117</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="63" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="19" t="s">
+      <c r="A15" s="18" t="s">
         <v>180</v>
       </c>
-      <c r="B15" s="19" t="s">
+      <c r="B15" s="18" t="s">
         <v>150</v>
       </c>
-      <c r="C15" s="19" t="s">
+      <c r="C15" s="18" t="s">
         <v>151</v>
       </c>
-      <c r="D15" s="19" t="s">
+      <c r="D15" s="18" t="s">
         <v>152</v>
       </c>
-      <c r="E15" s="19" t="s">
+      <c r="E15" s="18" t="s">
         <v>169</v>
       </c>
-      <c r="F15" s="19" t="s">
+      <c r="F15" s="18" t="s">
         <v>119</v>
       </c>
-      <c r="G15" s="19" t="s">
+      <c r="G15" s="18" t="s">
         <v>181</v>
       </c>
-      <c r="H15" s="19" t="s">
+      <c r="H15" s="18" t="s">
         <v>52</v>
       </c>
-      <c r="I15" s="24" t="n">
+      <c r="I15" s="23" t="n">
         <v>65000</v>
       </c>
-      <c r="J15" s="24" t="n">
+      <c r="J15" s="23" t="n">
         <v>80000</v>
       </c>
-      <c r="K15" s="20" t="n">
+      <c r="K15" s="19" t="n">
         <f aca="false">IF(I15="","",IFERROR(I15*INDEX(rates!$C$5:$C$12,MATCH($H15,rates!$A$5:$A$12,0)),"check currency code"))</f>
         <v>1235000</v>
       </c>
-      <c r="L15" s="20" t="n">
+      <c r="L15" s="19" t="n">
         <f aca="false">IF(J15="","",IFERROR(J15*INDEX(rates!$C$5:$C$12,MATCH($H15,rates!$A$5:$A$12,0)),"check currency code"))</f>
         <v>1520000</v>
       </c>
-      <c r="M15" s="25" t="n">
+      <c r="M15" s="24" t="n">
         <v>50</v>
       </c>
-      <c r="N15" s="25" t="n">
+      <c r="N15" s="24" t="n">
         <v>70</v>
       </c>
-      <c r="O15" s="25" t="n">
+      <c r="O15" s="28" t="n">
         <v>4</v>
       </c>
-      <c r="P15" s="26" t="s">
+      <c r="P15" s="25" t="s">
         <v>112</v>
       </c>
-      <c r="Q15" s="23" t="s">
+      <c r="Q15" s="22" t="s">
         <v>113</v>
       </c>
-      <c r="R15" s="21" t="s">
+      <c r="R15" s="20" t="s">
         <v>92</v>
       </c>
-      <c r="S15" s="28" t="s">
+      <c r="S15" s="21" t="s">
         <v>182</v>
       </c>
-      <c r="T15" s="19" t="s">
+      <c r="T15" s="18" t="s">
         <v>181</v>
       </c>
-      <c r="U15" s="28" t="n">
+      <c r="U15" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="V15" s="21" t="s">
+        <v>183</v>
+      </c>
+      <c r="W15" s="29" t="s">
+        <v>179</v>
+      </c>
+      <c r="X15" s="22" t="s">
+        <v>97</v>
+      </c>
+      <c r="Y15" s="17" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="21" t="s">
+        <v>184</v>
+      </c>
+      <c r="B16" s="21" t="s">
+        <v>185</v>
+      </c>
+      <c r="C16" s="21" t="s">
+        <v>185</v>
+      </c>
+      <c r="D16" s="21" t="s">
+        <v>186</v>
+      </c>
+      <c r="E16" s="21" t="s">
+        <v>187</v>
+      </c>
+      <c r="F16" s="21" t="s">
+        <v>188</v>
+      </c>
+      <c r="G16" s="21" t="s">
+        <v>189</v>
+      </c>
+      <c r="H16" s="21" t="s">
+        <v>56</v>
+      </c>
+      <c r="I16" s="27" t="n">
         <v>2</v>
       </c>
-      <c r="V15" s="28" t="s">
-        <v>183</v>
-      </c>
-      <c r="W15" s="31" t="s">
-        <v>179</v>
-      </c>
-      <c r="X15" s="23" t="s">
-        <v>97</v>
-      </c>
-      <c r="Y15" s="18" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="28" t="s">
-        <v>184</v>
-      </c>
-      <c r="B16" s="28" t="s">
-        <v>185</v>
-      </c>
-      <c r="C16" s="28" t="s">
-        <v>185</v>
-      </c>
-      <c r="D16" s="28" t="s">
-        <v>186</v>
-      </c>
-      <c r="E16" s="28" t="s">
-        <v>187</v>
-      </c>
-      <c r="F16" s="28" t="s">
-        <v>188</v>
-      </c>
-      <c r="G16" s="28" t="s">
-        <v>189</v>
-      </c>
-      <c r="H16" s="28" t="s">
-        <v>56</v>
-      </c>
-      <c r="I16" s="29" t="n">
-        <v>2</v>
-      </c>
-      <c r="J16" s="29" t="n">
+      <c r="J16" s="27" t="n">
         <v>2.5</v>
       </c>
-      <c r="K16" s="30" t="n">
+      <c r="K16" s="19" t="n">
         <f aca="false">IF(I16="","",IFERROR(I16*INDEX(rates!$C$5:$C$12,MATCH($H16,rates!$A$5:$A$12,0)),"check currency code"))</f>
         <v>39000</v>
       </c>
-      <c r="L16" s="30" t="n">
+      <c r="L16" s="19" t="n">
         <f aca="false">IF(J16="","",IFERROR(J16*INDEX(rates!$C$5:$C$12,MATCH($H16,rates!$A$5:$A$12,0)),"check currency code"))</f>
         <v>48750</v>
       </c>
-      <c r="M16" s="28" t="n">
+      <c r="M16" s="21" t="n">
         <v>35</v>
       </c>
-      <c r="N16" s="28" t="n">
+      <c r="N16" s="21" t="n">
         <v>50</v>
       </c>
-      <c r="O16" s="28" t="n">
-        <v>3</v>
-      </c>
-      <c r="P16" s="28" t="s">
+      <c r="O16" s="21" t="n">
+        <v>2</v>
+      </c>
+      <c r="P16" s="21" t="s">
         <v>90</v>
       </c>
-      <c r="Q16" s="23" t="s">
-        <v>141</v>
-      </c>
-      <c r="R16" s="23" t="s">
+      <c r="Q16" s="22" t="s">
         <v>190</v>
       </c>
-      <c r="S16" s="28" t="s">
+      <c r="R16" s="22" t="s">
         <v>191</v>
       </c>
-      <c r="T16" s="28" t="s">
+      <c r="S16" s="21" t="s">
+        <v>192</v>
+      </c>
+      <c r="T16" s="21" t="s">
         <v>94</v>
       </c>
-      <c r="U16" s="28" t="n">
+      <c r="U16" s="21" t="n">
         <v>1</v>
       </c>
-      <c r="V16" s="28" t="s">
-        <v>192</v>
-      </c>
-      <c r="W16" s="28" t="s">
+      <c r="V16" s="21" t="s">
         <v>193</v>
       </c>
-      <c r="X16" s="23" t="s">
+      <c r="W16" s="21" t="s">
+        <v>194</v>
+      </c>
+      <c r="X16" s="22" t="s">
         <v>97</v>
       </c>
-      <c r="Y16" s="18" t="s">
+      <c r="Y16" s="17" t="s">
         <v>98</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="28" t="s">
-        <v>194</v>
-      </c>
-      <c r="B17" s="28" t="s">
+      <c r="A17" s="21" t="s">
+        <v>195</v>
+      </c>
+      <c r="B17" s="21" t="s">
         <v>185</v>
       </c>
-      <c r="C17" s="28" t="s">
+      <c r="C17" s="21" t="s">
         <v>185</v>
       </c>
-      <c r="D17" s="28" t="s">
+      <c r="D17" s="21" t="s">
         <v>186</v>
       </c>
-      <c r="E17" s="28" t="s">
-        <v>195</v>
-      </c>
-      <c r="F17" s="28" t="s">
+      <c r="E17" s="21" t="s">
+        <v>196</v>
+      </c>
+      <c r="F17" s="21" t="s">
         <v>103</v>
       </c>
-      <c r="G17" s="28" t="s">
-        <v>196</v>
-      </c>
-      <c r="H17" s="28" t="s">
+      <c r="G17" s="21" t="s">
+        <v>197</v>
+      </c>
+      <c r="H17" s="21" t="s">
         <v>56</v>
       </c>
-      <c r="I17" s="29" t="n">
+      <c r="I17" s="27" t="n">
         <v>2</v>
       </c>
-      <c r="J17" s="29" t="n">
+      <c r="J17" s="27" t="n">
         <v>2.5</v>
       </c>
-      <c r="K17" s="30" t="n">
+      <c r="K17" s="19" t="n">
         <f aca="false">IF(I17="","",IFERROR(I17*INDEX(rates!$C$5:$C$12,MATCH($H17,rates!$A$5:$A$12,0)),"check currency code"))</f>
         <v>39000</v>
       </c>
-      <c r="L17" s="30" t="n">
+      <c r="L17" s="19" t="n">
         <f aca="false">IF(J17="","",IFERROR(J17*INDEX(rates!$C$5:$C$12,MATCH($H17,rates!$A$5:$A$12,0)),"check currency code"))</f>
         <v>48750</v>
       </c>
-      <c r="M17" s="28" t="n">
-        <v>60</v>
-      </c>
-      <c r="N17" s="28" t="n">
-        <v>80</v>
-      </c>
-      <c r="O17" s="28" t="n">
-        <v>1</v>
-      </c>
-      <c r="P17" s="28" t="s">
-        <v>197</v>
-      </c>
-      <c r="Q17" s="23" t="s">
+      <c r="M17" s="21" t="n">
+        <v>30</v>
+      </c>
+      <c r="N17" s="21" t="n">
+        <v>40</v>
+      </c>
+      <c r="O17" s="21" t="n">
+        <v>2</v>
+      </c>
+      <c r="P17" s="21" t="s">
+        <v>198</v>
+      </c>
+      <c r="Q17" s="22" t="s">
         <v>91</v>
       </c>
-      <c r="R17" s="23" t="s">
-        <v>198</v>
-      </c>
-      <c r="S17" s="28" t="s">
+      <c r="R17" s="22" t="s">
         <v>199</v>
       </c>
-      <c r="T17" s="28" t="s">
+      <c r="S17" s="21" t="s">
+        <v>200</v>
+      </c>
+      <c r="T17" s="21" t="s">
         <v>94</v>
       </c>
-      <c r="U17" s="28" t="n">
+      <c r="U17" s="21" t="n">
         <v>2</v>
       </c>
-      <c r="V17" s="28" t="s">
-        <v>200</v>
-      </c>
-      <c r="W17" s="28" t="s">
+      <c r="V17" s="21" t="s">
         <v>201</v>
       </c>
-      <c r="X17" s="23" t="s">
+      <c r="W17" s="21" t="s">
+        <v>202</v>
+      </c>
+      <c r="X17" s="22" t="s">
         <v>97</v>
       </c>
-      <c r="Y17" s="18" t="s">
+      <c r="Y17" s="17" t="s">
         <v>98</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="28" t="s">
-        <v>202</v>
-      </c>
-      <c r="B18" s="28" t="s">
+      <c r="A18" s="21" t="s">
+        <v>203</v>
+      </c>
+      <c r="B18" s="21" t="s">
         <v>185</v>
       </c>
-      <c r="C18" s="28" t="s">
+      <c r="C18" s="21" t="s">
         <v>185</v>
       </c>
-      <c r="D18" s="28" t="s">
+      <c r="D18" s="21" t="s">
         <v>186</v>
       </c>
-      <c r="E18" s="28" t="s">
+      <c r="E18" s="21" t="s">
         <v>187</v>
       </c>
-      <c r="F18" s="28" t="s">
+      <c r="F18" s="21" t="s">
         <v>110</v>
       </c>
-      <c r="G18" s="28" t="s">
-        <v>203</v>
-      </c>
-      <c r="H18" s="28" t="s">
+      <c r="G18" s="21" t="s">
+        <v>204</v>
+      </c>
+      <c r="H18" s="21" t="s">
         <v>56</v>
       </c>
-      <c r="I18" s="29" t="n">
-        <v>28</v>
-      </c>
-      <c r="J18" s="29" t="n">
-        <v>55</v>
-      </c>
-      <c r="K18" s="30" t="n">
+      <c r="I18" s="27" t="n">
+        <v>20</v>
+      </c>
+      <c r="J18" s="27" t="n">
+        <v>35</v>
+      </c>
+      <c r="K18" s="19" t="n">
         <f aca="false">IF(I18="","",IFERROR(I18*INDEX(rates!$C$5:$C$12,MATCH($H18,rates!$A$5:$A$12,0)),"check currency code"))</f>
-        <v>546000</v>
-      </c>
-      <c r="L18" s="30" t="n">
+        <v>390000</v>
+      </c>
+      <c r="L18" s="19" t="n">
         <f aca="false">IF(J18="","",IFERROR(J18*INDEX(rates!$C$5:$C$12,MATCH($H18,rates!$A$5:$A$12,0)),"check currency code"))</f>
-        <v>1072500</v>
-      </c>
-      <c r="M18" s="28" t="n">
-        <v>25</v>
-      </c>
-      <c r="N18" s="28" t="n">
+        <v>682500</v>
+      </c>
+      <c r="M18" s="21" t="n">
+        <v>15</v>
+      </c>
+      <c r="N18" s="21" t="n">
+        <v>30</v>
+      </c>
+      <c r="O18" s="21" t="n">
+        <v>4</v>
+      </c>
+      <c r="P18" s="21" t="s">
+        <v>112</v>
+      </c>
+      <c r="Q18" s="22" t="s">
+        <v>113</v>
+      </c>
+      <c r="R18" s="22" t="s">
+        <v>92</v>
+      </c>
+      <c r="S18" s="21" t="s">
+        <v>205</v>
+      </c>
+      <c r="T18" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="U18" s="21" t="n">
+        <v>2</v>
+      </c>
+      <c r="V18" s="21" t="s">
+        <v>206</v>
+      </c>
+      <c r="W18" s="21" t="s">
+        <v>207</v>
+      </c>
+      <c r="X18" s="22" t="s">
+        <v>97</v>
+      </c>
+      <c r="Y18" s="17" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="21" t="s">
+        <v>208</v>
+      </c>
+      <c r="B19" s="21" t="s">
+        <v>185</v>
+      </c>
+      <c r="C19" s="21" t="s">
+        <v>185</v>
+      </c>
+      <c r="D19" s="21" t="s">
+        <v>186</v>
+      </c>
+      <c r="E19" s="21" t="s">
+        <v>187</v>
+      </c>
+      <c r="F19" s="21" t="s">
+        <v>119</v>
+      </c>
+      <c r="G19" s="21" t="s">
+        <v>120</v>
+      </c>
+      <c r="H19" s="21" t="s">
+        <v>56</v>
+      </c>
+      <c r="I19" s="27" t="n">
+        <v>20</v>
+      </c>
+      <c r="J19" s="27" t="n">
         <v>40</v>
       </c>
-      <c r="O18" s="28" t="n">
-        <v>4</v>
-      </c>
-      <c r="P18" s="28" t="s">
-        <v>112</v>
-      </c>
-      <c r="Q18" s="23" t="s">
-        <v>113</v>
-      </c>
-      <c r="R18" s="23" t="s">
-        <v>92</v>
-      </c>
-      <c r="S18" s="28" t="s">
-        <v>204</v>
-      </c>
-      <c r="T18" s="28" t="s">
-        <v>94</v>
-      </c>
-      <c r="U18" s="28" t="n">
-        <v>2</v>
-      </c>
-      <c r="V18" s="28" t="s">
-        <v>205</v>
-      </c>
-      <c r="W18" s="28" t="s">
-        <v>206</v>
-      </c>
-      <c r="X18" s="23" t="s">
-        <v>97</v>
-      </c>
-      <c r="Y18" s="18" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="28" t="s">
-        <v>207</v>
-      </c>
-      <c r="B19" s="28" t="s">
-        <v>185</v>
-      </c>
-      <c r="C19" s="28" t="s">
-        <v>185</v>
-      </c>
-      <c r="D19" s="28" t="s">
-        <v>186</v>
-      </c>
-      <c r="E19" s="28" t="s">
-        <v>187</v>
-      </c>
-      <c r="F19" s="28" t="s">
-        <v>119</v>
-      </c>
-      <c r="G19" s="28" t="s">
-        <v>120</v>
-      </c>
-      <c r="H19" s="28" t="s">
-        <v>56</v>
-      </c>
-      <c r="I19" s="29" t="n">
-        <v>22</v>
-      </c>
-      <c r="J19" s="29" t="n">
-        <v>45</v>
-      </c>
-      <c r="K19" s="30" t="n">
+      <c r="K19" s="19" t="n">
         <f aca="false">IF(I19="","",IFERROR(I19*INDEX(rates!$C$5:$C$12,MATCH($H19,rates!$A$5:$A$12,0)),"check currency code"))</f>
-        <v>429000</v>
-      </c>
-      <c r="L19" s="30" t="n">
+        <v>390000</v>
+      </c>
+      <c r="L19" s="19" t="n">
         <f aca="false">IF(J19="","",IFERROR(J19*INDEX(rates!$C$5:$C$12,MATCH($H19,rates!$A$5:$A$12,0)),"check currency code"))</f>
-        <v>877500</v>
-      </c>
-      <c r="M19" s="28" t="n">
-        <v>25</v>
-      </c>
-      <c r="N19" s="28" t="n">
-        <v>40</v>
+        <v>780000</v>
+      </c>
+      <c r="M19" s="21" t="n">
+        <v>20</v>
+      </c>
+      <c r="N19" s="21" t="n">
+        <v>30</v>
       </c>
       <c r="O19" s="28" t="n">
         <v>4</v>
       </c>
-      <c r="P19" s="28" t="s">
+      <c r="P19" s="21" t="s">
         <v>112</v>
       </c>
-      <c r="Q19" s="23" t="s">
+      <c r="Q19" s="22" t="s">
         <v>113</v>
       </c>
-      <c r="R19" s="23" t="s">
+      <c r="R19" s="22" t="s">
         <v>92</v>
       </c>
-      <c r="S19" s="28" t="s">
-        <v>208</v>
-      </c>
-      <c r="T19" s="28" t="s">
+      <c r="S19" s="21" t="s">
+        <v>209</v>
+      </c>
+      <c r="T19" s="21" t="s">
         <v>120</v>
       </c>
-      <c r="U19" s="28" t="n">
+      <c r="U19" s="21" t="n">
         <v>1</v>
       </c>
-      <c r="V19" s="28" t="s">
-        <v>209</v>
-      </c>
-      <c r="W19" s="28" t="s">
+      <c r="V19" s="21" t="s">
         <v>210</v>
       </c>
-      <c r="X19" s="23" t="s">
+      <c r="W19" s="21" t="s">
+        <v>211</v>
+      </c>
+      <c r="X19" s="22" t="s">
         <v>97</v>
       </c>
-      <c r="Y19" s="18" t="s">
+      <c r="Y19" s="17" t="s">
         <v>117</v>
       </c>
     </row>

</xml_diff>